<commit_message>
update unit test plan with personal details
</commit_message>
<xml_diff>
--- a/Agile Documentation/Unit_Test_Plan_v0.1.xlsx
+++ b/Agile Documentation/Unit_Test_Plan_v0.1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://infosystechnologies-my.sharepoint.com/personal/kamaljeet_kaur01_ad_infosys_com1/Documents/Infosys/CC/Events/Oct 2021 - Mar 2022/CC2.0/Internship/Jan-Apr 2022/Artifacts/internship/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mallu\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3B9D4FEA-5A3F-460B-9A40-165575443B6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{23819564-CC70-4EEA-A2E6-76C4773036C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{C3B83BB6-2AB9-4547-8541-9F6969E92BF1}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C3B83BB6-2AB9-4547-8541-9F6969E92BF1}"/>
   </bookViews>
   <sheets>
     <sheet name="UT" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="27">
   <si>
     <t>Actual Result</t>
   </si>
@@ -52,6 +52,69 @@
   </si>
   <si>
     <t>Sl: No:</t>
+  </si>
+  <si>
+    <t>user Login &amp; Session Initialization</t>
+  </si>
+  <si>
+    <t>Enter valid user credentials on the login portal and submit.</t>
+  </si>
+  <si>
+    <t>Dtabase vertifiaction and Flask session token generation.</t>
+  </si>
+  <si>
+    <t>Successful authenticatioon and  redirection to the exam monitoring portal</t>
+  </si>
+  <si>
+    <t>passed</t>
+  </si>
+  <si>
+    <t>System accurately logs face-absent warning events into the database.</t>
+  </si>
+  <si>
+    <t>Haar Cascade classifier face frame tracking and absence interval logging</t>
+  </si>
+  <si>
+    <t>start the monitpring session and move the candidate's face away from the webcame</t>
+  </si>
+  <si>
+    <t>open cv face presence Detection</t>
+  </si>
+  <si>
+    <t>Tab switch/Focus Loss DETECTION</t>
+  </si>
+  <si>
+    <t>switchnto another browser tab or minimize the activate test window during</t>
+  </si>
+  <si>
+    <t>javascripts window blur and foucs event listeners.</t>
+  </si>
+  <si>
+    <t>Triggers and records integrity viiolations logs for tab switching.</t>
+  </si>
+  <si>
+    <t>Generates accurate risk scored and categorization n]metrics for the session.</t>
+  </si>
+  <si>
+    <t>pandas dataframe weighted penalty calculations and risk labeling</t>
+  </si>
+  <si>
+    <t>process accumulated session event logs throught yhe scoring modulel.</t>
+  </si>
+  <si>
+    <t>pandas integrity score calcu;ation</t>
+  </si>
+  <si>
+    <t>Dashboard Anlytics&amp;CSV/JSON Export test procedure</t>
+  </si>
+  <si>
+    <t>Naviagtie to the administartive streamlit dashboard and click export summary buttons</t>
+  </si>
+  <si>
+    <t>Dta visulaizations heatmaps rendering anf file download handles.</t>
+  </si>
+  <si>
+    <t>Dashboard displays metrics correctly and generates downloadable export files.</t>
   </si>
 </sst>
 </file>
@@ -444,16 +507,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF95B16C-182C-4757-B929-A728708A2DB0}">
   <dimension ref="A1:F6"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.140625" customWidth="1"/>
-    <col min="2" max="2" width="14.28515625" customWidth="1"/>
+    <col min="1" max="1" width="9.109375" customWidth="1"/>
+    <col min="2" max="2" width="14.33203125" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
-    <col min="4" max="5" width="16.5703125" customWidth="1"/>
-    <col min="6" max="6" width="15.85546875" customWidth="1"/>
+    <col min="4" max="5" width="16.5546875" customWidth="1"/>
+    <col min="6" max="6" width="15.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="31.5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" ht="31.2" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>5</v>
       </c>
@@ -473,45 +536,105 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A2" s="1"/>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
+    <row r="2" spans="1:6" ht="93.6" x14ac:dyDescent="0.25">
+      <c r="A2" s="1">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>10</v>
+      </c>
     </row>
-    <row r="3" spans="1:6" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
+    <row r="3" spans="1:6" ht="124.8" x14ac:dyDescent="0.25">
+      <c r="A3" s="1">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>10</v>
+      </c>
     </row>
-    <row r="4" spans="1:6" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A4" s="1"/>
-      <c r="B4" s="1"/>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1"/>
+    <row r="4" spans="1:6" ht="93.6" x14ac:dyDescent="0.25">
+      <c r="A4" s="1">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>10</v>
+      </c>
     </row>
-    <row r="5" spans="1:6" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A5" s="1"/>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
-      <c r="F5" s="1"/>
+    <row r="5" spans="1:6" ht="93.6" x14ac:dyDescent="0.25">
+      <c r="A5" s="1">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>10</v>
+      </c>
     </row>
-    <row r="6" spans="1:6" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A6" s="1"/>
-      <c r="B6" s="1"/>
-      <c r="C6" s="1"/>
-      <c r="D6" s="1"/>
-      <c r="E6" s="1"/>
-      <c r="F6" s="1"/>
+    <row r="6" spans="1:6" ht="140.4" x14ac:dyDescent="0.25">
+      <c r="A6" s="1">
+        <v>5</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>10</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>